<commit_message>
Add authentication, expense submission, approvals, and reports features
- Add Google OAuth login page and next-auth configuration
- Add expense creation page with AI-powered receipt analysis
- Add team approvals page for managers to approve/reject reports
- Add reports API with persistent JSON store (lib/reports-store.ts)
- Update submit-expenses route to save reports and support currency conversion
- Rename proxy.ts to middleware.ts for correct Next.js middleware resolution
- Replace NStarX logos with new Logo.png
- Clean up next.config.ts (remove ngrok dev origin)
- Update package.json with required dependencies (next-auth, nodemailer, exceljs)

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/app/data/employees.xlsx
+++ b/app/data/employees.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,12 +541,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Subbaraju</t>
+          <t>Nidhi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>subbaraju.chappidi@nstarxinc.com</t>
+          <t>nidhi.singh@nstarxinc.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -563,12 +563,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nidhi</t>
+          <t>Swaroopa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>nidhi.singh@nstarxinc.com</t>
+          <t>swaroopa.vanaparthi@nstarxinc.com</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -585,12 +585,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Swaroopa</t>
+          <t>Jabeen Khanam</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>swaroopa.vanaparthi@nstarxinc.com</t>
+          <t>jabeen.khanam@nstarxinc.com</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -607,12 +607,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Dosala Shiva Shankaraiah</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>saiteja.ramagiri@nstarxinc.com</t>
+          <t>shiva.dosala@nstarxinc.com</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -629,12 +629,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Smruthi Kothakonda</t>
+          <t>Thota Naresh</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>smruthi.kothakonda@nstarxinc.com</t>
+          <t>naresh.thota@nstarxinc.com</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -651,12 +651,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sravani Koukuntla</t>
+          <t>Ashok Munagala</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>sravani.koukuntla@nstarxinc.com</t>
+          <t>ashok.munagala@nstarxinc.com</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -673,12 +673,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jabeen Khanam</t>
+          <t>Sai Srinivas Potla</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>jabeen.khanam@nstarxinc.com</t>
+          <t>saisrinivas.potla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -695,12 +695,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rajan Kumar </t>
+          <t>Naresh Sowoju</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>rajan.sharma@nstarxinc.com</t>
+          <t>naresh.sowoju@nstarxinc.com</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -717,12 +717,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Dosala Shiva Shankaraiah</t>
+          <t>Geethika Kakarla</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>shiva.dosala@nstarxinc.com</t>
+          <t>geethika.kakarla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -739,12 +739,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Arun Goluguri</t>
+          <t>Narayana Reddy Bogireddy</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>arun.goluguri@nstarxinc.com</t>
+          <t>narayana.bogireddy@nstarxinc.com</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -761,12 +761,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Saketh Dahagam</t>
+          <t>Apparao Buddha</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>saketh.dahagam@nstarxinc.com</t>
+          <t>apparao.buddha@nstarxinc.com</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -783,12 +783,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>M Veena Madhuri</t>
+          <t>Ganesh Vallamla</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">veena.motupalli@nstarxinc.com </t>
+          <t>ganesh.vallamla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -805,12 +805,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Naveen Babu Yarlagadda</t>
+          <t>Venkat Murthy Velamala</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>yarlagadda@nstarxinc.com</t>
+          <t>venkat.velamala@nstarxinc.com</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -827,12 +827,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Nagasandeep Motupalli</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sandeep.motupalli@nstarxinc.com</t>
+          <t>tapas.acharjee@nstarxinc.com</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -849,17 +849,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Shravan Kumar A S</t>
+          <t>Mohd Khaja Shujauddin</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>shravan.kumar@nstarxinc.com</t>
+          <t>khaja.shujauddin@nstarxinc.com</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -871,17 +871,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hariteja  Eeraparaju</t>
+          <t>Tejaswani Kambampati</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>hariteja.eeraparaju@nstarxinc.com</t>
+          <t>tejaswini.kambampati@nstarxinc.com</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -893,17 +893,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Suresh Goparaju</t>
+          <t>Keertipati Chandu Varma</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>suresh.goparaju@nstarxinc.com</t>
+          <t>chandu.keertipati@nstarxinc.com</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -915,17 +915,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Venkat Pogakula</t>
+          <t>Chandana Gidugu</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>venkat.pogakula@nstarxinc.com</t>
+          <t>chandana.gidugu@nstarxinc.com</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -937,17 +937,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Thota Naresh</t>
+          <t>Prajakta Shikare Maruti</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>naresh.thota@nstarxinc.com</t>
+          <t>prajakta.shikare@nstarxinc.com</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -959,17 +959,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ashok Munagala</t>
+          <t>Amar Sai Veeravalli</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ashok.munagala@nstarxinc.com</t>
+          <t>amar.veeravalli@nstarxinc.com</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -981,17 +981,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sampath Gattu</t>
+          <t>Sai Krishna Andhavarapu</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>sampath.gattu@nstarxinc.com</t>
+          <t>saikrishna.andhavarapu@nstarxinc.com</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1003,39 +1003,39 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Deepak Devaraj</t>
+          <t>Anveshitha Thota</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>deepak.devaraj@nstarxinc.com</t>
+          <t>anveshitha.thota@nstarxinc.com</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Sai Srinivas Potla</t>
+          <t>Bera Sireesha Krishnaveni</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>saisrinivas.potla@nstarxinc.com</t>
+          <t>sireesha.bera@nstarxinc.com</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Smruthi Kothakonda</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1047,17 +1047,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Naresh Sowoju</t>
+          <t>Ramesh Bevara</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>naresh.sowoju@nstarxinc.com</t>
+          <t>ramesh.bevara@nstarxinc.com</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Uday kiran Y</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1069,17 +1069,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Geethika Kakarla</t>
+          <t>Rajeshwar</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>geethika.kakarla@nstarxinc.com</t>
+          <t>rajeshwar.bommena@nstarxinc.com</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Syam Sundar Devarakonda</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1091,17 +1091,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Narayana Reddy Bogireddy</t>
+          <t>Pramod Kumar Kodoju</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>narayana.bogireddy@nstarxinc.com</t>
+          <t>pramod.kodoju@nstarxinc.com</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Syam Sundar Devarakonda</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1113,17 +1113,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Apparao Buddha</t>
+          <t>Younus Shaik</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>apparao.buddha@nstarxinc.com</t>
+          <t>younus.shaik@nstarxinc.com</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Syam Sundar Devarakonda</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1135,17 +1135,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ganesh Vallamla</t>
+          <t>Babita Kumar</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ganesh.vallamla@nstarxinc.com</t>
+          <t>babita.kumar@nstarxinc.com</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Syam Sundar Devarakonda</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1157,61 +1157,61 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Venkat Murthy Velamala</t>
+          <t>Jesus Fernandez</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>venkat.velamala@nstarxinc.com</t>
+          <t>jesus.fernandez@nstarxinc.com</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Syam Sundar Devarakonda</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Spain</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Chaitanya Dhanalakota</t>
+          <t>Ganesh Tyagali</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>chaitanya.dhanalakota@nstarxinc.com</t>
+          <t xml:space="preserve">ganesh.tyagali@nstarxinc.com </t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Angshuman Patra</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Tapas Kumar Acharjee</t>
+          <t>Syam Sundar Devarakonda</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>tapas.acharjee@nstarxinc.com</t>
+          <t>syamsundar.devarakonda@nstarxinc.com</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Amol  Patalay</t>
+          <t>Angshuman Patra</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1223,127 +1223,127 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tejaswini Kande</t>
+          <t>Suman Kalyan</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>tejaswini.kande@nstarxinc.com</t>
+          <t>suman.kalyan@nstarxinc.com</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Angshuman Patra</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Spain</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Sirisha Achnala</t>
+          <t>Dakshina Murthy Karra</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>sirisha.achnala@nstarxinc.com</t>
+          <t>dakshinamurthy.karra@nstarxinc.com</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Angshuman Patra</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Siva Reddy Evuri</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>siva.evuri@nstarxinc.com</t>
+          <t>sujay@nstarxinc.com</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Angshuman Patra</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Kotla Pavani Priyanka</t>
+          <t>Adrian Paleacu</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>pavani.kotla@nstarxinc.com</t>
+          <t>adrian.paleacu@nstarxinc.com</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Suman Kalyan</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Romania</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SwamiNaidu Seepana</t>
+          <t>Gabriel Trautmann</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>swaminaidu.seepana@nstarxinc.com</t>
+          <t>gabriel.trautmann@nstarxinc.com</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Suman Kalyan</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Romania</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Raghava Harshavardhan Raju</t>
+          <t>Sneha Sahu</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>harshavardhan.raghava@nstarxinc.com</t>
+          <t>sneha.sahu@nstarxinc.com</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1355,17 +1355,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Shashank Illa</t>
+          <t>Vaibhav Mittal</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>shashank.illa@nstarxinc.com</t>
+          <t>vaibhav.mittal@nstarxinc.com</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Subbaraju Chappidi</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1377,17 +1377,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mohd Khaja Shujauddin</t>
+          <t>Nikhil Sham Vanjari</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>khaja.shujauddin@nstarxinc.com</t>
+          <t>nikhil.vanjari@nstarxinc.com</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1399,17 +1399,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tejaswani Kambampati</t>
+          <t>Kontham Anand kumar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>tejaswini.kambampati@nstarxinc.com</t>
+          <t>anand.kontham@nstarxinc.com</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1421,17 +1421,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Keertipati Chandu Varma</t>
+          <t>Shriyans Kandhagatla</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>chandu.keertipati@nstarxinc.com</t>
+          <t>shriyans.kandhagatla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1443,17 +1443,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Chandana Gidugu</t>
+          <t>Arya Pulkit</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>chandana.gidugu@nstarxinc.com</t>
+          <t>arya.pulkit@nstarxinc.com</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1465,39 +1465,39 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Prajakta Shikare Maruti</t>
+          <t>Britney H</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>prajakta.shikare@nstarxinc.com</t>
+          <t>britney@nstarxinc.com</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Amar Sai Veeravalli</t>
+          <t>Sai Vyvaswath Bhupasamudram</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>amar.veeravalli@nstarxinc.com</t>
+          <t>saivyvaswath.bhupasamudram@nstarxinc.com</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1509,17 +1509,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sai Krishna Andhavarapu</t>
+          <t>Kriti Bhagat</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>saikrishna.andhavarapu@nstarxinc.com</t>
+          <t>kriti.bhagat@nstarxinc.com</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1531,17 +1531,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Anveshitha Thota</t>
+          <t>Debopriyo Ghosh</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>anveshitha.thota@nstarxinc.com</t>
+          <t>debopriyo.ghosh@nstarxinc.com</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ramagiri Saiteja</t>
+          <t>Sujikar Reddy Varidireddy</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1553,17 +1553,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nuty Vanitha</t>
+          <t>K Anjali Achary</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>vanitha.nuty@nstarxinc.com</t>
+          <t>anjali.kottapalli@nstarxinc.com</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Smruthi Kothakonda</t>
+          <t>Younus Shaik</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1575,17 +1575,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Devadula Sai Sudheer</t>
+          <t>M Veena Madhuri</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>sudheer.devadula@nstarxinc.com</t>
+          <t xml:space="preserve">veena.motupalli@nstarxinc.com </t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Smruthi Kothakonda</t>
+          <t>M Veena Madhuri</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1597,17 +1597,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Gouni Saideepthi</t>
+          <t>Shantanu Chaturvedi</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>saideepthi.gouni@nstarxinc.com</t>
+          <t>shantanu.chaturvedi@nstarxinc.com</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Smruthi Kothakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1619,39 +1619,39 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bera Sireesha Krishnaveni</t>
+          <t>Sidharth Kondapuram</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>sireesha.bera@nstarxinc.com</t>
+          <t>sidharth.kondapuram@nstarxinc.com</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Smruthi Kothakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Spain</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Venkata Lalitha Suresh Emani</t>
+          <t>Navdeep Singh</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>suresh.emani@nstarxinc.com</t>
+          <t>kevin.singh@nstarx.com</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Uday kiran Y</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1663,17 +1663,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Sindhu Pogula</t>
+          <t>Jhanvi Sharma</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>sindhu.pogula@nstarxinc.com</t>
+          <t>Jenny.white@nstarxinc.com</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Uday kiran Y</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1685,17 +1685,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Ramesh Bevara</t>
+          <t>Saloni Singh Andotra</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ramesh.bevara@nstarxinc.com</t>
+          <t>stephany@nstarxinc.com</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Uday kiran Y</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1707,17 +1707,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Rajeshwar</t>
+          <t>Anchal Bakshi</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>rajeshwar.bommena@nstarxinc.com</t>
+          <t>alice.williams@nstarxinc.com</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Syam Sundar Devarakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -1729,17 +1729,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Pramod Kumar Kodoju</t>
+          <t>Sarika Sharma</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>pramod.kodoju@nstarxinc.com</t>
+          <t>shelly.mccullam@nstarxinc.com</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Syam Sundar Devarakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -1751,17 +1751,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Younus Shaik</t>
+          <t>MN Prasad Reddy</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>younus.shaik@nstarxinc.com</t>
+          <t>prasad.reddy@nstarxinc.com</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Syam Sundar Devarakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1773,127 +1773,127 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Babita Kumar</t>
+          <t>Chris Hundertmark</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>babita.kumar@nstarxinc.com</t>
+          <t>chris.hundertmark@nstarxinc.com</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Syam Sundar Devarakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Jesus Fernandez</t>
+          <t>Joseph Caponsacco</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>jesus.fernandez@nstarxinc.com</t>
+          <t>joseph.caponsacco@nstarxinc.com</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Syam Sundar Devarakonda</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ganesh Tyagali</t>
+          <t>Nikita Sharma</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">ganesh.tyagali@nstarxinc.com </t>
+          <t>nancy.miller@nstarxinc.com</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Angshuman Patra</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Syam Sundar Devarakonda</t>
+          <t>Shuaib Noori</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>syamsundar.devarakonda@nstarxinc.com</t>
+          <t>shuaib.noori@nstarxinc.com</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Angshuman Patra</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Suman Kalyan</t>
+          <t>Urja Bhandari</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>suman.kalyan@nstarxinc.com</t>
+          <t>una.jones@nstarxinc.com</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Angshuman Patra</t>
+          <t>Sujay Kumar</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Dakshina Murthy Karra</t>
+          <t>Sachin Chaudhari</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>dakshinamurthy.karra@nstarxinc.com</t>
+          <t>sachin.chaudhari@nstarxinc.com</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Angshuman Patra</t>
+          <t>Shayne Pinto</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -1905,83 +1905,83 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>sujay@nstarxinc.com</t>
+          <t>ramakrishna.bellum@nstarxinc.com</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Angshuman Patra</t>
+          <t>Shayne Pinto</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Adrian Paleacu</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>adrian.paleacu@nstarxinc.com</t>
+          <t>mohin.shaik@nstarxinc.com</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Suman Kalyan</t>
+          <t>Shayne Pinto</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Gabriel Trautmann</t>
+          <t>Abhirupa Sen</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>gabriel.trautmann@nstarxinc.com</t>
+          <t>abhirupa.sen@nstarxinc.com</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Suman Kalyan</t>
+          <t>Shayne Pinto</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Sneha Sahu</t>
+          <t>Bommadevara Kavyabharathi</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>sneha.sahu@nstarxinc.com</t>
+          <t>kavya.bommadevara@nstarxinc.com</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -1993,17 +1993,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Vaibhav Mittal</t>
+          <t>Kotturi Supriya</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>vaibhav.mittal@nstarxinc.com</t>
+          <t>supriya.kotturi@nstarxinc.com</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2015,17 +2015,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Nikhil Sham Vanjari</t>
+          <t>Sai Shiva Naga Gudla</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>nikhil.vanjari@nstarxinc.com</t>
+          <t>saishiva.gudla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2037,17 +2037,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Kontham Anand kumar</t>
+          <t>Sanket Khushal Patil</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>anand.kontham@nstarxinc.com</t>
+          <t>sanket.patil@nstarxinc.com</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2059,17 +2059,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Shriyans Kandhagatla</t>
+          <t>Vikram Dattatray Danvale</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>shriyans.kandhagatla@nstarxinc.com</t>
+          <t>vikram.danvale@nstarxinc.com</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2081,17 +2081,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Arya Pulkit</t>
+          <t>Rishi Soni</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>arya.pulkit@nstarxinc.com</t>
+          <t>rishi.soni@nstarxinc.com</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -2103,39 +2103,39 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Britney H</t>
+          <t>Akunuri Jai Tiru Ganesh</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>britney@nstarxinc.com</t>
+          <t>jai.akunuri@nstarxinc.com</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Sai Vyvaswath Bhupasamudram</t>
+          <t>Suneel Kumar Reddy Vaka</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>saivyvaswath.bhupasamudram@nstarxinc.com</t>
+          <t>suneel.vaka@nstarxinc.com</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2147,17 +2147,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Kriti Bhagat</t>
+          <t>Manish Gari</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>kriti.bhagat@nstarxinc.com</t>
+          <t xml:space="preserve">manish.gari@nstarxinc.com </t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2169,39 +2169,39 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Debopriyo Ghosh</t>
+          <t>Yassir Benhammou</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>debopriyo.ghosh@nstarxinc.com</t>
+          <t xml:space="preserve">yassir.benhammou@nstarxinc.com </t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Sujikar Reddy Varidireddy</t>
+          <t>Bellum Sai Siva Rama Krishna</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Spain</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>K Anjali Achary</t>
+          <t>Uday kiran Y</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>anjali.kottapalli@nstarxinc.com</t>
+          <t>uday.kiran@nstarxinc.com</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Younus Shaik</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2213,17 +2213,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Shantanu Chaturvedi</t>
+          <t>Rohit Kumar</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>shantanu.chaturvedi@nstarxinc.com</t>
+          <t>rohit.kumar@nstarxinc.com</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2235,39 +2235,39 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Sidharth Kondapuram</t>
+          <t>Venkata Santosh Krishna Teja Ghanta</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>sidharth.kondapuram@nstarxinc.com</t>
+          <t>santosh.ghanta@nstarxinc.com</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Navdeep Singh</t>
+          <t>Inguva Satyavenkata Sai Kumar</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>kevin.singh@nstarx.com</t>
+          <t>sai.inguva@nstarxinc.com</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2279,17 +2279,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Jhanvi Sharma</t>
+          <t>Chowdarapu Srivatsa</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Jenny.white@nstarxinc.com</t>
+          <t>srivatsa.chowdarapu@nstarxinc.com</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2301,17 +2301,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Saloni Singh Andotra</t>
+          <t>Heet Hiteshkumar Gorakhiya</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>stephany@nstarxinc.com</t>
+          <t>heet.gorakhiya@nstarxinc.com</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2323,17 +2323,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Anchal Bakshi</t>
+          <t>Shaurya Prakash Singh</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>alice.williams@nstarxinc.com</t>
+          <t>shaurya.singh@nstarxinc.com</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2345,17 +2345,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Sarika Sharma</t>
+          <t>Rahul Holekeri</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>shelly.mccullam@nstarxinc.com</t>
+          <t>rahul.holikeri@nstarxinc.com</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2367,17 +2367,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>MN Prasad Reddy</t>
+          <t>Suresh Babu Konapuram</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>prasad.reddy@nstarxinc.com</t>
+          <t>konapuram@nstarxinc.com</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2389,61 +2389,61 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Chris Hundertmark</t>
+          <t>Alessandro Tiberio</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>chris.hundertmark@nstarxinc.com</t>
+          <t>alessandro.tiberio@nstarxinc.com</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>Spain</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Joseph Caponsacco</t>
+          <t>Sowmya Kunapuli</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>joseph.caponsacco@nstarxinc.com</t>
+          <t>sowmya.kunapuli@nstarxinc.com</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Nikita Sharma</t>
+          <t>Raju Pasunuri</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>nancy.miller@nstarxinc.com</t>
+          <t>raju.pasunuri@nstarxinc.com</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Sujay Kumar</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2455,39 +2455,39 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Sachin Chaudhari</t>
+          <t>Sriram Narayan</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>sachin.chaudhari@nstarxinc.com</t>
+          <t>sriram.narayan@nstarxinc.com</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Shayne Pinto</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Ayush Kumar</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ramakrishna.bellum@nstarxinc.com</t>
+          <t>ayush.kumar@nstarxinc.com</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Shayne Pinto</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -2499,17 +2499,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>Gurunath Kamale</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>gurunath.kamale@nstarxinc.com</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
           <t>Mohin Shaik</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>mohin.shaik@nstarxinc.com</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Shayne Pinto</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -2521,39 +2521,39 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Abhirupa Sen</t>
+          <t>Srigiri Sai Manish</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>abhirupa.sen@nstarxinc.com</t>
+          <t>manish.srigiri@nstarxinc.com</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Shayne Pinto</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Bommadevara Kavyabharathi</t>
+          <t>Vaishnavi Anaboina</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>kavya.bommadevara@nstarxinc.com</t>
+          <t>vaishnavi.anaboina@nstarxinc.com</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -2565,17 +2565,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Kotturi Supriya</t>
+          <t>Krishnamurty Kotikalapudi</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>supriya.kotturi@nstarxinc.com</t>
+          <t>krishnamurty.kotikalapudi@nstarxinc.com</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -2587,17 +2587,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Sai Shiva Naga Gudla</t>
+          <t>Dakshith Gundapuneni</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>saishiva.gudla@nstarxinc.com</t>
+          <t>dakshith.gundapuneni@nstarxinc.com</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -2609,17 +2609,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Sanket Khushal Patil</t>
+          <t>Divya Sinha</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>sanket.patil@nstarxinc.com</t>
+          <t>divya.sinha@nstarxinc.com</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Mohin Shaik</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -2631,17 +2631,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Vikram Dattatray Danvale</t>
+          <t>Subbaraju</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>vikram.danvale@nstarxinc.com</t>
+          <t>subbaraju.chappidi@nstarxinc.com</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -2653,17 +2653,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Rishi Soni</t>
+          <t>Ramagiri Saiteja</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>rishi.soni@nstarxinc.com</t>
+          <t>saiteja.ramagiri@nstarxinc.com</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -2675,17 +2675,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Akunuri Jai Tiru Ganesh</t>
+          <t>Nuty Vanitha</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>jai.akunuri@nstarxinc.com</t>
+          <t>vanitha.nuty@nstarxinc.com</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -2697,17 +2697,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Suneel Kumar Reddy Vaka</t>
+          <t>Smruthi Kothakonda</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>suneel.vaka@nstarxinc.com</t>
+          <t>smruthi.kothakonda@nstarxinc.com</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -2719,17 +2719,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Manish Gari</t>
+          <t>Sravani Koukuntla</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">manish.gari@nstarxinc.com </t>
+          <t>sravani.koukuntla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -2741,39 +2741,39 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Yassir Benhammou</t>
+          <t>Tejaswini Kande</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">yassir.benhammou@nstarxinc.com </t>
+          <t>tejaswini.kande@nstarxinc.com</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Bellum Sai Siva Rama Krishna</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Uday kiran Y</t>
+          <t>Sirisha Achnala</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>uday.kiran@nstarxinc.com</t>
+          <t>sirisha.achnala@nstarxinc.com</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -2785,17 +2785,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Rohit Kumar</t>
+          <t>Siva Reddy Evuri</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>rohit.kumar@nstarxinc.com</t>
+          <t>siva.evuri@nstarxinc.com</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -2807,17 +2807,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Venkata Santosh Krishna Teja Ghanta</t>
+          <t>Devadula Sai Sudheer</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>santosh.ghanta@nstarxinc.com</t>
+          <t>sudheer.devadula@nstarxinc.com</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -2829,17 +2829,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Inguva Satyavenkata Sai Kumar</t>
+          <t>Venkata Lalitha Suresh Emani</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>sai.inguva@nstarxinc.com</t>
+          <t>suresh.emani@nstarxinc.com</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -2851,17 +2851,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Chowdarapu Srivatsa</t>
+          <t xml:space="preserve">Rajan Kumar </t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>srivatsa.chowdarapu@nstarxinc.com</t>
+          <t>rajan.sharma@nstarxinc.com</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -2873,17 +2873,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Heet Hiteshkumar Gorakhiya</t>
+          <t>Sindhu Pogula</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>heet.gorakhiya@nstarxinc.com</t>
+          <t>sindhu.pogula@nstarxinc.com</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -2895,17 +2895,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Shaurya Prakash Singh</t>
+          <t>Kotla Pavani Priyanka</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>shaurya.singh@nstarxinc.com</t>
+          <t>pavani.kotla@nstarxinc.com</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -2917,17 +2917,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Rahul Holekeri</t>
+          <t>SwamiNaidu Seepana</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>rahul.holikeri@nstarxinc.com</t>
+          <t>swaminaidu.seepana@nstarxinc.com</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -2939,17 +2939,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Suresh Babu Konapuram</t>
+          <t>Raghava Harshavardhan Raju</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>konapuram@nstarxinc.com</t>
+          <t>harshavardhan.raghava@nstarxinc.com</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -2961,39 +2961,39 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Alessandro Tiberio</t>
+          <t>Gouni Saideepthi</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>alessandro.tiberio@nstarxinc.com</t>
+          <t>saideepthi.gouni@nstarxinc.com</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>India</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Sowmya Kunapuli</t>
+          <t>Saketh Dahagam</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>sowmya.kunapuli@nstarxinc.com</t>
+          <t>saketh.dahagam@nstarxinc.com</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3005,17 +3005,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Raju Pasunuri</t>
+          <t>Naveen Babu Yarlagadda</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>raju.pasunuri@nstarxinc.com</t>
+          <t>yarlagadda@nstarxinc.com</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3027,17 +3027,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Sriram Narayan</t>
+          <t>Nagasandeep Motupalli</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>sriram.narayan@nstarxinc.com</t>
+          <t>sandeep.motupalli@nstarxinc.com</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3049,17 +3049,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Ayush Kumar</t>
+          <t>Shravan Kumar A S</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>ayush.kumar@nstarxinc.com</t>
+          <t>shravan.kumar@nstarxinc.com</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -3071,17 +3071,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Gurunath Kamale</t>
+          <t>Hariteja  Eeraparaju</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>gurunath.kamale@nstarxinc.com</t>
+          <t>hariteja.eeraparaju@nstarxinc.com</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3093,17 +3093,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Srigiri Sai Manish</t>
+          <t>Suresh Goparaju</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>manish.srigiri@nstarxinc.com</t>
+          <t>suresh.goparaju@nstarxinc.com</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -3115,17 +3115,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Vaishnavi Anaboina</t>
+          <t>Venkat Pogakula</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>vaishnavi.anaboina@nstarxinc.com</t>
+          <t>venkat.pogakula@nstarxinc.com</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -3137,17 +3137,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Krishnamurty Kotikalapudi</t>
+          <t>Sampath Gattu</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>krishnamurty.kotikalapudi@nstarxinc.com</t>
+          <t>sampath.gattu@nstarxinc.com</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -3159,42 +3159,64 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Dakshith Gundapuneni</t>
+          <t>Deepak Devaraj</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>dakshith.gundapuneni@nstarxinc.com</t>
+          <t>deepak.devaraj@nstarxinc.com</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>US</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Divya Sinha</t>
+          <t>Chaitanya Dhanalakota</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>divya.sinha@nstarxinc.com</t>
+          <t>chaitanya.dhanalakota@nstarxinc.com</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Mohin Shaik</t>
+          <t>Tapas Kumar Acharjee</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Shashank Illa</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>shashank.illa@nstarxinc.com</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Tapas Kumar Acharjee</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
         <is>
           <t>India</t>
         </is>

</xml_diff>